<commit_message>
fine tune model with linear/ridge regression and strength of schedule
</commit_message>
<xml_diff>
--- a/Rankings.xlsx
+++ b/Rankings.xlsx
@@ -451,11 +451,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Big Sur</t>
+          <t>Massachusetts</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>34.375</v>
+        <v>47.85922756360216</v>
       </c>
     </row>
     <row r="3">
@@ -464,11 +464,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>Baton Rouge</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>32.625</v>
+        <v>46.77161685233727</v>
       </c>
     </row>
     <row r="4">
@@ -477,11 +477,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Minnesota</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>32.58823529411764</v>
+        <v>46.53973287018938</v>
       </c>
     </row>
     <row r="5">
@@ -490,11 +490,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Massachusetts</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>32.55555555555556</v>
+        <v>46.17168217369726</v>
       </c>
     </row>
     <row r="6">
@@ -503,11 +503,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Big Sur</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>31.375</v>
+        <v>44.04555507464867</v>
       </c>
     </row>
     <row r="7">
@@ -516,11 +516,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Illinois</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>29.88235294117647</v>
+        <v>43.6923691331897</v>
       </c>
     </row>
     <row r="8">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>29.77777777777778</v>
+        <v>41.31013363790528</v>
       </c>
     </row>
     <row r="9">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>28.77777777777778</v>
+        <v>40.35518865220078</v>
       </c>
     </row>
     <row r="10">
@@ -555,11 +555,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Baton Rouge</t>
+          <t>Boise</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>27.76470588235295</v>
+        <v>36.93365168946455</v>
       </c>
     </row>
     <row r="11">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>26.625</v>
+        <v>32.12282228635277</v>
       </c>
     </row>
     <row r="12">
@@ -581,11 +581,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>25.64705882352942</v>
+        <v>31.63583216701932</v>
       </c>
     </row>
     <row r="13">
@@ -594,11 +594,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Illinois</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>24.47058823529412</v>
+        <v>30.73691112158542</v>
       </c>
     </row>
     <row r="14">
@@ -607,11 +607,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>22.82352941176471</v>
+        <v>30.34429174057223</v>
       </c>
     </row>
     <row r="15">
@@ -620,11 +620,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>21.2</v>
+        <v>28.95298705882353</v>
       </c>
     </row>
     <row r="16">
@@ -633,11 +633,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Key Largo</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>19.75</v>
+        <v>28.92296890950663</v>
       </c>
     </row>
     <row r="17">
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>19.5</v>
+        <v>28.41904055992057</v>
       </c>
     </row>
     <row r="18">
@@ -659,11 +659,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Boise</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>19.05882352941176</v>
+        <v>27.83777674139889</v>
       </c>
     </row>
     <row r="19">
@@ -672,11 +672,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18.58823529411765</v>
+        <v>26.02503184101846</v>
       </c>
     </row>
     <row r="20">
@@ -685,11 +685,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Belgrade</t>
+          <t>Madison</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17.76470588235294</v>
+        <v>25.90189768600079</v>
       </c>
     </row>
     <row r="21">
@@ -698,11 +698,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Osaka</t>
+          <t>Augusta</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>16.70588235294118</v>
+        <v>25.37469783349331</v>
       </c>
     </row>
     <row r="22">
@@ -711,11 +711,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>New Hope</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>16.35294117647059</v>
+        <v>25.19547056402887</v>
       </c>
     </row>
     <row r="23">
@@ -724,11 +724,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Trenton</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>16.23529411764706</v>
+        <v>24.57540316759317</v>
       </c>
     </row>
     <row r="24">
@@ -737,11 +737,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Juneau</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>15.76470588235294</v>
+        <v>24.51052687760176</v>
       </c>
     </row>
     <row r="25">
@@ -750,11 +750,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>South Dakota</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>15.73333333333333</v>
+        <v>23.77640235294118</v>
       </c>
     </row>
     <row r="26">
@@ -763,11 +763,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Providence</t>
+          <t>Mississippi</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>15.375</v>
+        <v>23.15889267216349</v>
       </c>
     </row>
     <row r="27">
@@ -776,11 +776,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>New Hope</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>15.22222222222222</v>
+        <v>23.09536935480986</v>
       </c>
     </row>
     <row r="28">
@@ -789,11 +789,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>NYC</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>14.82352941176471</v>
+        <v>23.06187348388663</v>
       </c>
     </row>
     <row r="29">
@@ -802,11 +802,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Helena</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>14</v>
+        <v>22.19183212258819</v>
       </c>
     </row>
     <row r="30">
@@ -815,11 +815,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Concord</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>13.88888888888889</v>
+        <v>21.85286181640051</v>
       </c>
     </row>
     <row r="31">
@@ -828,11 +828,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Madison</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>13.88235294117647</v>
+        <v>21.59870830212039</v>
       </c>
     </row>
     <row r="32">
@@ -841,11 +841,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>New Jersey</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>13.6</v>
+        <v>21.32122352941177</v>
       </c>
     </row>
     <row r="33">
@@ -854,11 +854,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Fort Worth</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>13.52941176470588</v>
+        <v>20.40505962695348</v>
       </c>
     </row>
     <row r="34">
@@ -867,11 +867,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Nantucket</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>13.1764705882353</v>
+        <v>19.9906647477059</v>
       </c>
     </row>
     <row r="35">
@@ -880,11 +880,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Dover</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>13.06666666666667</v>
+        <v>19.64681254211945</v>
       </c>
     </row>
     <row r="36">
@@ -893,11 +893,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Belgrade</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>12.35294117647059</v>
+        <v>19.40770470588236</v>
       </c>
     </row>
     <row r="37">
@@ -906,11 +906,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Juneau</t>
+          <t>Colorado</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>12.25</v>
+        <v>19.2176365253341</v>
       </c>
     </row>
     <row r="38">
@@ -919,11 +919,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mississippi</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>11.88888888888889</v>
+        <v>18.93559125239375</v>
       </c>
     </row>
     <row r="39">
@@ -932,11 +932,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>11.88235294117647</v>
+        <v>18.27316235294118</v>
       </c>
     </row>
     <row r="40">
@@ -945,11 +945,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>11.76470588235294</v>
+        <v>18.20594705882353</v>
       </c>
     </row>
     <row r="41">
@@ -958,11 +958,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Connecticut</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>11.375</v>
+        <v>15.88329170895858</v>
       </c>
     </row>
     <row r="42">
@@ -971,11 +971,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>11.375</v>
+        <v>15.62888988700425</v>
       </c>
     </row>
     <row r="43">
@@ -984,11 +984,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Key Largo</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>10.875</v>
+        <v>15.39619335173398</v>
       </c>
     </row>
     <row r="44">
@@ -997,11 +997,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Fort Worth</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>10.58823529411765</v>
+        <v>15.03661176470589</v>
       </c>
     </row>
     <row r="45">
@@ -1010,11 +1010,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Augusta</t>
+          <t>England</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>10.58823529411765</v>
+        <v>14.86794588235294</v>
       </c>
     </row>
     <row r="46">
@@ -1023,11 +1023,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>New Hampshire</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>10.5</v>
+        <v>14.77400133385311</v>
       </c>
     </row>
     <row r="47">
@@ -1036,11 +1036,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>10</v>
+        <v>14.06679895740059</v>
       </c>
     </row>
     <row r="48">
@@ -1049,11 +1049,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Nantucket</t>
+          <t>Natchez</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9.625</v>
+        <v>13.76064368500169</v>
       </c>
     </row>
     <row r="49">
@@ -1062,11 +1062,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Iceland</t>
+          <t>Topeka</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>9.411764705882353</v>
+        <v>13.73170482958078</v>
       </c>
     </row>
     <row r="50">
@@ -1075,11 +1075,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Bismarck</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>8.823529411764707</v>
+        <v>13.6634988221932</v>
       </c>
     </row>
     <row r="51">
@@ -1088,11 +1088,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>8.266666666666666</v>
+        <v>13.41564588235294</v>
       </c>
     </row>
     <row r="52">
@@ -1101,11 +1101,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Vermont</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>8.23529411764706</v>
+        <v>13.02703301774186</v>
       </c>
     </row>
     <row r="53">
@@ -1114,11 +1114,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>8.117647058823531</v>
+        <v>12.66033764705883</v>
       </c>
     </row>
     <row r="54">
@@ -1127,11 +1127,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Topeka</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>7.75</v>
+        <v>11.98213145530528</v>
       </c>
     </row>
     <row r="55">
@@ -1140,11 +1140,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Delaware</t>
+          <t>Alaska</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>7.375</v>
+        <v>11.64636149271445</v>
       </c>
     </row>
     <row r="56">
@@ -1153,11 +1153,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Annapolis</t>
+          <t>Ohio</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>6.875</v>
+        <v>10.08170267584319</v>
       </c>
     </row>
     <row r="57">
@@ -1166,11 +1166,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>Osaka</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>6.823529411764706</v>
+        <v>9.770677647058825</v>
       </c>
     </row>
     <row r="58">
@@ -1179,11 +1179,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>London</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>6.705882352941177</v>
+        <v>9.683483529411767</v>
       </c>
     </row>
     <row r="59">
@@ -1192,11 +1192,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>6.625</v>
+        <v>9.235285882352944</v>
       </c>
     </row>
     <row r="60">
@@ -1205,11 +1205,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Prague</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>6.23529411764706</v>
+        <v>9.180304705882357</v>
       </c>
     </row>
     <row r="61">
@@ -1218,11 +1218,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Des Moines</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>6</v>
+        <v>9.164720601561401</v>
       </c>
     </row>
     <row r="62">
@@ -1231,11 +1231,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>El Paso</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>6</v>
+        <v>7.975801349617646</v>
       </c>
     </row>
     <row r="63">
@@ -1244,11 +1244,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Idaho</t>
+          <t>Annapolis</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>6</v>
+        <v>7.922776983539976</v>
       </c>
     </row>
     <row r="64">
@@ -1257,11 +1257,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Concord</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>5.75</v>
+        <v>7.705386927033494</v>
       </c>
     </row>
     <row r="65">
@@ -1270,11 +1270,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>5.625</v>
+        <v>7.466467058823532</v>
       </c>
     </row>
     <row r="66">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>5.625</v>
+        <v>7.385127781001968</v>
       </c>
     </row>
     <row r="67">
@@ -1296,11 +1296,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Trenton</t>
+          <t>Olympia</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>5.5</v>
+        <v>7.349521045161709</v>
       </c>
     </row>
     <row r="68">
@@ -1309,11 +1309,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Michigan</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>5.176470588235294</v>
+        <v>7.260866284023402</v>
       </c>
     </row>
     <row r="69">
@@ -1322,11 +1322,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Montana</t>
+          <t>Frankfort</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>5.066666666666666</v>
+        <v>7.254234114480527</v>
       </c>
     </row>
     <row r="70">
@@ -1335,11 +1335,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>5.058823529411765</v>
+        <v>6.282874117647061</v>
       </c>
     </row>
     <row r="71">
@@ -1348,11 +1348,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Bismarck</t>
+          <t>Saint Paul</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>4.875</v>
+        <v>6.06297627795306</v>
       </c>
     </row>
     <row r="72">
@@ -1361,11 +1361,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>Hartford</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>4.625</v>
+        <v>5.348354150291534</v>
       </c>
     </row>
     <row r="73">
@@ -1374,11 +1374,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Prague</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4.000000000000001</v>
+        <v>4.947609411764708</v>
       </c>
     </row>
     <row r="74">
@@ -1387,11 +1387,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Florence</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>4.000000000000001</v>
+        <v>4.296615294117649</v>
       </c>
     </row>
     <row r="75">
@@ -1400,11 +1400,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Providence</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>4</v>
+        <v>4.010966145678688</v>
       </c>
     </row>
     <row r="76">
@@ -1413,11 +1413,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>4</v>
+        <v>3.93529577435876</v>
       </c>
     </row>
     <row r="77">
@@ -1426,11 +1426,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Louisiana</t>
+          <t>Delaware</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3.882352941176471</v>
+        <v>3.575053887514612</v>
       </c>
     </row>
     <row r="78">
@@ -1439,11 +1439,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Wilmington</t>
+          <t>Indiana</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3.375</v>
+        <v>3.53587539418811</v>
       </c>
     </row>
     <row r="79">
@@ -1452,11 +1452,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>California</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3.333333333333333</v>
+        <v>2.910607515312666</v>
       </c>
     </row>
     <row r="80">
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3.176470588235294</v>
+        <v>2.781707058823531</v>
       </c>
     </row>
     <row r="81">
@@ -1478,11 +1478,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Lincoln</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2.933333333333334</v>
+        <v>2.460858152595841</v>
       </c>
     </row>
     <row r="82">
@@ -1491,11 +1491,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Alaska</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2.375</v>
+        <v>2.443870416608533</v>
       </c>
     </row>
     <row r="83">
@@ -1504,11 +1504,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Vermont</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2.25</v>
+        <v>2.284328594346955</v>
       </c>
     </row>
     <row r="84">
@@ -1517,11 +1517,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1.625</v>
+        <v>2.219518868875639</v>
       </c>
     </row>
     <row r="85">
@@ -1530,11 +1530,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Lincoln</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1.5</v>
+        <v>2.112130588235296</v>
       </c>
     </row>
     <row r="86">
@@ -1543,11 +1543,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Hartford</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1.411764705882353</v>
+        <v>2.07578207350403</v>
       </c>
     </row>
     <row r="87">
@@ -1556,11 +1556,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Venice</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1.25</v>
+        <v>0.9492964705882361</v>
       </c>
     </row>
     <row r="88">
@@ -1569,11 +1569,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Des Moines</t>
+          <t>Lakeland</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.6061159444898614</v>
       </c>
     </row>
     <row r="89">
@@ -1582,11 +1582,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>0.875</v>
+        <v>0.307093509248114</v>
       </c>
     </row>
     <row r="90">
@@ -1595,11 +1595,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>Istanbul</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.2096070588235309</v>
       </c>
     </row>
     <row r="91">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Florence</t>
+          <t>New Jersey</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>0.5882352941176471</v>
+        <v>-0.5448285257927505</v>
       </c>
     </row>
     <row r="92">
@@ -1621,11 +1621,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>New Hampshire</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>0.5882352941176471</v>
+        <v>-0.6824776810648725</v>
       </c>
     </row>
     <row r="93">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Istanbul</t>
+          <t>Hawaii</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>0.4705882352941176</v>
+        <v>-0.9897833748768541</v>
       </c>
     </row>
     <row r="94">
@@ -1647,11 +1647,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Harrisburg</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>-0.375</v>
+        <v>-1.476081376943956</v>
       </c>
     </row>
     <row r="95">
@@ -1660,11 +1660,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Princeton</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>-0.5882352941176471</v>
+        <v>-1.754889621583196</v>
       </c>
     </row>
     <row r="96">
@@ -1673,11 +1673,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>El Paso</t>
+          <t>Iceland</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>-1.058823529411765</v>
+        <v>-1.934101176470589</v>
       </c>
     </row>
     <row r="97">
@@ -1686,11 +1686,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>-1.125</v>
+        <v>-2.27445176470588</v>
       </c>
     </row>
     <row r="98">
@@ -1699,11 +1699,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Venice</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>-1.294117647058824</v>
+        <v>-2.855297663536536</v>
       </c>
     </row>
     <row r="99">
@@ -1712,11 +1712,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Raleigh</t>
+          <t>Beijing</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>-1.294117647058824</v>
+        <v>-4.492324705882353</v>
       </c>
     </row>
     <row r="100">
@@ -1725,11 +1725,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Dover</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>-1.333333333333333</v>
+        <v>-4.770717647058821</v>
       </c>
     </row>
     <row r="101">
@@ -1738,11 +1738,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Colorado</t>
+          <t>Oklahoma</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>-1.75</v>
+        <v>-4.916404611708877</v>
       </c>
     </row>
     <row r="102">
@@ -1751,11 +1751,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Natchez</t>
+          <t>South Dakota</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>-1.875</v>
+        <v>-5.826426373547182</v>
       </c>
     </row>
     <row r="103">
@@ -1764,11 +1764,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Lansing</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>-2.117647058823529</v>
+        <v>-5.889559011794827</v>
       </c>
     </row>
     <row r="104">
@@ -1777,11 +1777,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>-2.375</v>
+        <v>-6.181121388316851</v>
       </c>
     </row>
     <row r="105">
@@ -1790,11 +1790,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Frankfort</t>
+          <t>Washington</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>-2.625</v>
+        <v>-6.788263615731108</v>
       </c>
     </row>
     <row r="106">
@@ -1803,11 +1803,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>West Virginia</t>
+          <t>Idaho</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>-2.75</v>
+        <v>-7.07810635267691</v>
       </c>
     </row>
     <row r="107">
@@ -1816,11 +1816,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Wyoming</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>-3.5</v>
+        <v>-7.102545559529756</v>
       </c>
     </row>
     <row r="108">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Nevada</t>
+          <t>Cheyenne</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>-3.6</v>
+        <v>-7.319984020368508</v>
       </c>
     </row>
     <row r="109">
@@ -1842,11 +1842,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>-4</v>
+        <v>-7.872815981364202</v>
       </c>
     </row>
     <row r="110">
@@ -1855,11 +1855,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Olympia</t>
+          <t>Connecticut</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>-4.235294117647059</v>
+        <v>-8.109173891895363</v>
       </c>
     </row>
     <row r="111">
@@ -1868,11 +1868,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>-4.625</v>
+        <v>-8.317627058823529</v>
       </c>
     </row>
     <row r="112">
@@ -1881,11 +1881,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Ohio</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>-4.875</v>
+        <v>-9.110398421616894</v>
       </c>
     </row>
     <row r="113">
@@ -1894,11 +1894,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Harrisburg</t>
+          <t>Shenzhen</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>-5.125</v>
+        <v>-9.166062352941177</v>
       </c>
     </row>
     <row r="114">
@@ -1907,11 +1907,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Wilmington</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>-5.375</v>
+        <v>-9.910863422764894</v>
       </c>
     </row>
     <row r="115">
@@ -1920,11 +1920,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Helena</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>-5.625</v>
+        <v>-10.22531233637883</v>
       </c>
     </row>
     <row r="116">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Louisiana</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>-6.124999999999999</v>
+        <v>-10.29437575076427</v>
       </c>
     </row>
     <row r="117">
@@ -1946,11 +1946,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Beijing</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>-6.352941176470589</v>
+        <v>-10.53323667276475</v>
       </c>
     </row>
     <row r="118">
@@ -1959,11 +1959,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Madrid</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>-6.5</v>
+        <v>-11.57273411764706</v>
       </c>
     </row>
     <row r="119">
@@ -1972,11 +1972,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Shenzhen</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>-6.588235294117648</v>
+        <v>-11.8617439055852</v>
       </c>
     </row>
     <row r="120">
@@ -1985,11 +1985,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Rhode Island</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>-7.125</v>
+        <v>-12.34332272768591</v>
       </c>
     </row>
     <row r="121">
@@ -1998,11 +1998,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Montpelier</t>
+          <t>Alabama</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>-7.466666666666666</v>
+        <v>-13.23757512811225</v>
       </c>
     </row>
     <row r="122">
@@ -2011,11 +2011,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>New Mexico</t>
+          <t>Oregon</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>-8.375</v>
+        <v>-13.40269103437803</v>
       </c>
     </row>
     <row r="123">
@@ -2024,11 +2024,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>New Mexico</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>-8.823529411764707</v>
+        <v>-14.60873360371722</v>
       </c>
     </row>
     <row r="124">
@@ -2037,11 +2037,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>Utah</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>-9.25</v>
+        <v>-17.77992558839047</v>
       </c>
     </row>
     <row r="125">
@@ -2050,11 +2050,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>-10</v>
+        <v>-17.79932235294118</v>
       </c>
     </row>
     <row r="126">
@@ -2063,11 +2063,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>Lansing</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>-10</v>
+        <v>-17.87413583618724</v>
       </c>
     </row>
     <row r="127">
@@ -2076,11 +2076,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Nevada</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>-10.25</v>
+        <v>-17.91283879771879</v>
       </c>
     </row>
     <row r="128">
@@ -2089,11 +2089,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Oregon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>-11.52941176470588</v>
+        <v>-18.22896102326664</v>
       </c>
     </row>
     <row r="129">
@@ -2102,11 +2102,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Saint Paul</t>
+          <t>Cape Coral</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>-12.5</v>
+        <v>-18.83088429265389</v>
       </c>
     </row>
     <row r="130">
@@ -2115,11 +2115,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Albany</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>-13.29411764705882</v>
+        <v>-19.23659135092024</v>
       </c>
     </row>
     <row r="131">
@@ -2128,11 +2128,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Lakeland</t>
+          <t>Wyoming</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>-14.75</v>
+        <v>-20.07927833977772</v>
       </c>
     </row>
     <row r="132">
@@ -2141,11 +2141,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-15.05882352941176</v>
+        <v>-20.09472632138812</v>
       </c>
     </row>
     <row r="133">
@@ -2154,11 +2154,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Cheyenne</t>
+          <t>Jefferson City</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>-15.375</v>
+        <v>-20.67724618646479</v>
       </c>
     </row>
     <row r="134">
@@ -2167,11 +2167,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Salem</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-15.625</v>
+        <v>-20.85387551099291</v>
       </c>
     </row>
     <row r="135">
@@ -2180,11 +2180,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Missouri</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-15.64705882352941</v>
+        <v>-20.92863345457658</v>
       </c>
     </row>
     <row r="136">
@@ -2193,11 +2193,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-15.75</v>
+        <v>-21.77215239690846</v>
       </c>
     </row>
     <row r="137">
@@ -2206,11 +2206,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Hawaii</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>-16.375</v>
+        <v>-22.11309058823529</v>
       </c>
     </row>
     <row r="138">
@@ -2219,11 +2219,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Princeton</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-17</v>
+        <v>-22.33730458059103</v>
       </c>
     </row>
     <row r="139">
@@ -2236,7 +2236,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-17.73333333333333</v>
+        <v>-22.43878131853511</v>
       </c>
     </row>
     <row r="140">
@@ -2245,11 +2245,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Albany</t>
+          <t>Montana</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-17.875</v>
+        <v>-23.22868817814706</v>
       </c>
     </row>
     <row r="141">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Springfield</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-18.125</v>
+        <v>-23.88701934321472</v>
       </c>
     </row>
     <row r="142">
@@ -2271,11 +2271,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>-18.25</v>
+        <v>-24.26231248419238</v>
       </c>
     </row>
     <row r="143">
@@ -2284,11 +2284,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Raleigh</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>-18.25</v>
+        <v>-25.49047539819689</v>
       </c>
     </row>
     <row r="144">
@@ -2297,11 +2297,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Rome</t>
+          <t>North Dakota</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>-18.94117647058824</v>
+        <v>-26.35695380609137</v>
       </c>
     </row>
     <row r="145">
@@ -2310,11 +2310,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Maryland</t>
+          <t>Pierre</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>-19.625</v>
+        <v>-27.6725745881087</v>
       </c>
     </row>
     <row r="146">
@@ -2323,11 +2323,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>North Dakota</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>-19.75</v>
+        <v>-28.73889051455351</v>
       </c>
     </row>
     <row r="147">
@@ -2336,11 +2336,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Cape Coral</t>
+          <t>Montpelier</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>-22.375</v>
+        <v>-29.07129380537339</v>
       </c>
     </row>
     <row r="148">
@@ -2349,11 +2349,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Rhode Island</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>-22.70588235294118</v>
+        <v>-29.59718097585165</v>
       </c>
     </row>
     <row r="149">
@@ -2362,11 +2362,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Oklahoma</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>-23.625</v>
+        <v>-29.59991294117647</v>
       </c>
     </row>
     <row r="150">
@@ -2375,11 +2375,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>West Virginia</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>-25.25</v>
+        <v>-29.83608542897511</v>
       </c>
     </row>
     <row r="151">
@@ -2388,11 +2388,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>South Carolina</t>
+          <t>Shanghai</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>-25.625</v>
+        <v>-31.11385647058824</v>
       </c>
     </row>
     <row r="152">
@@ -2405,7 +2405,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>-25.88235294117647</v>
+        <v>-31.63041529411765</v>
       </c>
     </row>
     <row r="153">
@@ -2414,11 +2414,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>-27.29411764705882</v>
+        <v>-32.10351936386154</v>
       </c>
     </row>
     <row r="154">
@@ -2427,11 +2427,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Sedona</t>
+          <t>Salem</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>-27.375</v>
+        <v>-32.37804917414272</v>
       </c>
     </row>
     <row r="155">
@@ -2440,11 +2440,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Maryland</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>-27.41176470588236</v>
+        <v>-33.06427113594142</v>
       </c>
     </row>
     <row r="156">
@@ -2453,11 +2453,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Maine</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>-27.52941176470588</v>
+        <v>-34.94394235294118</v>
       </c>
     </row>
     <row r="157">
@@ -2466,11 +2466,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>-27.625</v>
+        <v>-35.51911696022204</v>
       </c>
     </row>
     <row r="158">
@@ -2479,11 +2479,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Montgomery</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>-32.47058823529412</v>
+        <v>-35.55886738947892</v>
       </c>
     </row>
     <row r="159">
@@ -2492,11 +2492,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Jefferson City</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>-33.875</v>
+        <v>-37.84702998482265</v>
       </c>
     </row>
     <row r="160">
@@ -2505,11 +2505,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Shanghai</t>
+          <t>Bangkok</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>-34</v>
+        <v>-43.10546823529412</v>
       </c>
     </row>
     <row r="161">
@@ -2518,11 +2518,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Carson City</t>
+          <t>Maine</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>-34.66666666666666</v>
+        <v>-43.40563789535055</v>
       </c>
     </row>
     <row r="162">
@@ -2531,11 +2531,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>South Carolina</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>-35.29411764705883</v>
+        <v>-45.00104337751019</v>
       </c>
     </row>
     <row r="163">
@@ -2544,11 +2544,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Montgomery</t>
+          <t>Sedona</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>-35.33333333333333</v>
+        <v>-45.21224597171278</v>
       </c>
     </row>
     <row r="164">
@@ -2557,11 +2557,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Carson City</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>-39.875</v>
+        <v>-47.5648934123202</v>
       </c>
     </row>
     <row r="165">
@@ -2574,7 +2574,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>-42</v>
+        <v>-47.96620430625501</v>
       </c>
     </row>
     <row r="166">
@@ -2583,11 +2583,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>-45.76470588235294</v>
+        <v>-50.9609194412477</v>
       </c>
     </row>
   </sheetData>

</xml_diff>